<commit_message>
Vague 4 : vingt-quatre exercices, et la documentation à jour
Les quinze catégories restées à un exercice par notion sont relevées. Le ratio
minimal passe de 1,00 à 1,25, la médiane de 1,33 à 1,40 : plus aucune
catégorie n'est au plancher.

253 exercices, 246 définitions, 90,5 h, 1 497 téléchargements.

Deux défauts d'outillage corrigés au passage. Le chargeur des vagues de
lots.py tenait une liste de modules à la main — la septième du projet — et
découvre désormais. Et mes fonctions utilitaires s'appelaient _f et _b : en
IronPython 2, la variable de boucle d'une compréhension fuit dans la portée
englobante et les écrasait, d'où « bool is not callable ». Troisième fois que
ce piège se referme ; les noms courts sont désormais réservés aux boucles.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fondamentaux Grasshopper - IndC - 01-09-2026.xlsx
+++ b/Fondamentaux Grasshopper - IndC - 01-09-2026.xlsx
@@ -210,11 +210,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="Q6" s="10" t="inlineStr">
         <is>
-          <t>RH-01, RH-11</t>
+          <t>RH-01, RH-11, RH-30</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="Q7" s="10" t="inlineStr">
         <is>
-          <t>RH-02, RH-13</t>
+          <t>RH-02, RH-13, RH-30</t>
         </is>
       </c>
     </row>
@@ -1522,14 +1522,14 @@
       <c r="M8" s="7" t="inlineStr"/>
       <c r="N8" s="8" t="inlineStr"/>
       <c r="O8" s="10" t="inlineStr"/>
-      <c r="P8" s="12" t="inlineStr">
-        <is>
-          <t>Connaissance</t>
+      <c r="P8" s="11" t="inlineStr">
+        <is>
+          <t>Compétence</t>
         </is>
       </c>
       <c r="Q8" s="10" t="inlineStr">
         <is>
-          <t>RH-06</t>
+          <t>RH-06, RH-31</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="Q9" s="10" t="inlineStr">
         <is>
-          <t>RH-02, RH-13</t>
+          <t>RH-02, RH-13, RH-31</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="Q10" s="10" t="inlineStr">
         <is>
-          <t>RH-03</t>
+          <t>RH-03, RH-27</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="Q11" s="10" t="inlineStr">
         <is>
-          <t>RH-03, RH-14</t>
+          <t>RH-03, RH-14, RH-27</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="Q12" s="10" t="inlineStr">
         <is>
-          <t>RH-04, RH-15</t>
+          <t>RH-04, RH-15, RH-28</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="Q13" s="10" t="inlineStr">
         <is>
-          <t>RH-04, RH-16</t>
+          <t>RH-04, RH-16, RH-28</t>
         </is>
       </c>
     </row>
@@ -1919,7 +1919,7 @@
       </c>
       <c r="Q14" s="10" t="inlineStr">
         <is>
-          <t>RH-04, RH-16</t>
+          <t>RH-04, RH-16, RH-28</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="Q15" s="10" t="inlineStr">
         <is>
-          <t>RH-05, RH-17</t>
+          <t>RH-05, RH-17, RH-29</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="Q16" s="10" t="inlineStr">
         <is>
-          <t>RH-03, RH-14</t>
+          <t>RH-03, RH-14, RH-29</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="Q17" s="10" t="inlineStr">
         <is>
-          <t>RH-02</t>
+          <t>RH-02, RH-32</t>
         </is>
       </c>
     </row>
@@ -2172,14 +2172,14 @@
       <c r="M18" s="7" t="inlineStr"/>
       <c r="N18" s="8" t="inlineStr"/>
       <c r="O18" s="10" t="inlineStr"/>
-      <c r="P18" s="12" t="inlineStr">
-        <is>
-          <t>Connaissance</t>
+      <c r="P18" s="11" t="inlineStr">
+        <is>
+          <t>Compétence</t>
         </is>
       </c>
       <c r="Q18" s="10" t="inlineStr">
         <is>
-          <t>RH-07</t>
+          <t>RH-07, RH-32</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="Q19" s="10" t="inlineStr">
         <is>
-          <t>RH-23</t>
+          <t>RH-23, RH-32</t>
         </is>
       </c>
     </row>
@@ -2309,7 +2309,7 @@
       </c>
       <c r="Q20" s="10" t="inlineStr">
         <is>
-          <t>RH-09, RH-18</t>
+          <t>RH-09, RH-18, RH-24</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="Q21" s="10" t="inlineStr">
         <is>
-          <t>RH-07, RH-19</t>
+          <t>RH-07, RH-19, RH-24</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="Q22" s="10" t="inlineStr">
         <is>
-          <t>RH-09, RH-19</t>
+          <t>RH-09, RH-19, RH-24</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="Q23" s="10" t="inlineStr">
         <is>
-          <t>RH-08, RH-20</t>
+          <t>RH-08, RH-20, RH-25</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2569,7 @@
       </c>
       <c r="Q24" s="10" t="inlineStr">
         <is>
-          <t>RH-08, RH-20</t>
+          <t>RH-08, RH-20, RH-25</t>
         </is>
       </c>
     </row>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="Q25" s="10" t="inlineStr">
         <is>
-          <t>RH-08, RH-20</t>
+          <t>RH-08, RH-20, RH-25</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="Q26" s="10" t="inlineStr">
         <is>
-          <t>RH-08, RH-21</t>
+          <t>RH-08, RH-21, RH-26</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="Q27" s="10" t="inlineStr">
         <is>
-          <t>RH-08, RH-21</t>
+          <t>RH-08, RH-21, RH-26</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="Q28" s="10" t="inlineStr">
         <is>
-          <t>RH-10, RH-22</t>
+          <t>RH-10, RH-22, RH-26</t>
         </is>
       </c>
     </row>
@@ -2842,12 +2842,12 @@
           <t>REF-025</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>Principes et interface Grasshopper</t>
         </is>
@@ -2887,7 +2887,7 @@
       <c r="M29" s="7" t="inlineStr"/>
       <c r="N29" s="8" t="inlineStr"/>
       <c r="O29" s="10" t="inlineStr"/>
-      <c r="P29" s="12" t="inlineStr">
+      <c r="P29" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -2907,12 +2907,12 @@
           <t>REF-026</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Principes et interface Grasshopper</t>
         </is>
@@ -2972,12 +2972,12 @@
           <t>REF-027</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>Principes et interface Grasshopper</t>
         </is>
@@ -3037,12 +3037,12 @@
           <t>REF-028</t>
         </is>
       </c>
-      <c r="C32" s="13" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D32" s="13" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>Principes et interface Grasshopper</t>
         </is>
@@ -3102,12 +3102,12 @@
           <t>REF-029</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3154,7 +3154,7 @@
       </c>
       <c r="Q33" s="10" t="inlineStr">
         <is>
-          <t>PL-02, PL-05, PL-10</t>
+          <t>PL-02, PL-05, PL-10, PL-13, PL-16</t>
         </is>
       </c>
     </row>
@@ -3167,12 +3167,12 @@
           <t>REF-030</t>
         </is>
       </c>
-      <c r="C34" s="13" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="Q34" s="10" t="inlineStr">
         <is>
-          <t>PL-02, PL-05, PL-09, PL-10</t>
+          <t>PL-02, PL-05, PL-09, PL-10, PL-13</t>
         </is>
       </c>
     </row>
@@ -3232,12 +3232,12 @@
           <t>REF-031</t>
         </is>
       </c>
-      <c r="C35" s="13" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="Q35" s="10" t="inlineStr">
         <is>
-          <t>PL-03, PL-08, PL-11</t>
+          <t>PL-03, PL-08, PL-11, PL-14</t>
         </is>
       </c>
     </row>
@@ -3297,12 +3297,12 @@
           <t>REF-032</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3349,7 +3349,7 @@
       </c>
       <c r="Q36" s="10" t="inlineStr">
         <is>
-          <t>PL-03, PL-08</t>
+          <t>PL-03, PL-08, PL-14</t>
         </is>
       </c>
     </row>
@@ -3362,12 +3362,12 @@
           <t>REF-033</t>
         </is>
       </c>
-      <c r="C37" s="13" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D37" s="13" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="Q37" s="10" t="inlineStr">
         <is>
-          <t>PL-03, PL-08</t>
+          <t>PL-03, PL-08, PL-14</t>
         </is>
       </c>
     </row>
@@ -3427,12 +3427,12 @@
           <t>REF-034</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="D38" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="Q38" s="10" t="inlineStr">
         <is>
-          <t>PL-03, PL-11</t>
+          <t>PL-03, PL-11, PL-14</t>
         </is>
       </c>
     </row>
@@ -3492,12 +3492,12 @@
           <t>REF-035</t>
         </is>
       </c>
-      <c r="C39" s="13" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D39" s="13" t="inlineStr">
+      <c r="D39" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3544,7 +3544,7 @@
       </c>
       <c r="Q39" s="10" t="inlineStr">
         <is>
-          <t>PL-03, PL-11</t>
+          <t>PL-03, PL-11, PL-14</t>
         </is>
       </c>
     </row>
@@ -3557,12 +3557,12 @@
           <t>REF-036</t>
         </is>
       </c>
-      <c r="C40" s="13" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="D40" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="Q40" s="10" t="inlineStr">
         <is>
-          <t>PL-03, PL-11</t>
+          <t>PL-03, PL-11, PL-14</t>
         </is>
       </c>
     </row>
@@ -3622,12 +3622,12 @@
           <t>REF-037</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D41" s="13" t="inlineStr">
+      <c r="D41" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="Q41" s="10" t="inlineStr">
         <is>
-          <t>PL-03, PL-11</t>
+          <t>PL-03, PL-11, PL-14</t>
         </is>
       </c>
     </row>
@@ -3687,12 +3687,12 @@
           <t>REF-038</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="Q42" s="10" t="inlineStr">
         <is>
-          <t>PL-04, PL-06, PL-07</t>
+          <t>PL-04, PL-06, PL-07, PL-15, PL-16</t>
         </is>
       </c>
     </row>
@@ -3752,12 +3752,12 @@
           <t>REF-039</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C43" s="12" t="inlineStr">
         <is>
           <t>2 – Environnement et principes Grasshopper</t>
         </is>
       </c>
-      <c r="D43" s="13" t="inlineStr">
+      <c r="D43" s="12" t="inlineStr">
         <is>
           <t>Écosystème de plugins</t>
         </is>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="Q43" s="10" t="inlineStr">
         <is>
-          <t>PL-04, PL-06, PL-07, PL-12</t>
+          <t>PL-04, PL-06, PL-07, PL-12, PL-15, PL-16</t>
         </is>
       </c>
     </row>
@@ -6278,7 +6278,7 @@
       </c>
       <c r="Q81" s="10" t="inlineStr">
         <is>
-          <t>GP-02</t>
+          <t>GP-02, GP-13</t>
         </is>
       </c>
     </row>
@@ -6336,14 +6336,14 @@
       <c r="M82" s="7" t="inlineStr"/>
       <c r="N82" s="8" t="inlineStr"/>
       <c r="O82" s="10" t="inlineStr"/>
-      <c r="P82" s="12" t="inlineStr">
-        <is>
-          <t>Connaissance</t>
+      <c r="P82" s="11" t="inlineStr">
+        <is>
+          <t>Compétence</t>
         </is>
       </c>
       <c r="Q82" s="10" t="inlineStr">
         <is>
-          <t>GP-10</t>
+          <t>GP-10, GP-13</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="Q83" s="10" t="inlineStr">
         <is>
-          <t>GP-11</t>
+          <t>GP-11, GP-13</t>
         </is>
       </c>
     </row>
@@ -7636,7 +7636,7 @@
       <c r="M102" s="7" t="inlineStr"/>
       <c r="N102" s="8" t="inlineStr"/>
       <c r="O102" s="10" t="inlineStr"/>
-      <c r="P102" s="12" t="inlineStr">
+      <c r="P102" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -7701,7 +7701,7 @@
       <c r="M103" s="7" t="inlineStr"/>
       <c r="N103" s="8" t="inlineStr"/>
       <c r="O103" s="10" t="inlineStr"/>
-      <c r="P103" s="12" t="inlineStr">
+      <c r="P103" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -8091,7 +8091,7 @@
       <c r="M109" s="7" t="inlineStr"/>
       <c r="N109" s="8" t="inlineStr"/>
       <c r="O109" s="10" t="inlineStr"/>
-      <c r="P109" s="12" t="inlineStr">
+      <c r="P109" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -8221,7 +8221,7 @@
       <c r="M111" s="7" t="inlineStr"/>
       <c r="N111" s="8" t="inlineStr"/>
       <c r="O111" s="10" t="inlineStr"/>
-      <c r="P111" s="12" t="inlineStr">
+      <c r="P111" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -8871,7 +8871,7 @@
       <c r="M121" s="7" t="inlineStr"/>
       <c r="N121" s="8" t="inlineStr"/>
       <c r="O121" s="10" t="inlineStr"/>
-      <c r="P121" s="12" t="inlineStr">
+      <c r="P121" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -9203,7 +9203,7 @@
       </c>
       <c r="Q126" s="10" t="inlineStr">
         <is>
-          <t>WB-02</t>
+          <t>WB-02, WB-11</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="Q127" s="10" t="inlineStr">
         <is>
-          <t>WB-02, WB-06</t>
+          <t>WB-02, WB-06, WB-11</t>
         </is>
       </c>
     </row>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="Q128" s="10" t="inlineStr">
         <is>
-          <t>WB-02, WB-07</t>
+          <t>WB-02, WB-07, WB-11</t>
         </is>
       </c>
     </row>
@@ -9391,14 +9391,14 @@
       <c r="M129" s="7" t="inlineStr"/>
       <c r="N129" s="8" t="inlineStr"/>
       <c r="O129" s="10" t="inlineStr"/>
-      <c r="P129" s="12" t="inlineStr">
-        <is>
-          <t>Connaissance</t>
+      <c r="P129" s="11" t="inlineStr">
+        <is>
+          <t>Compétence</t>
         </is>
       </c>
       <c r="Q129" s="10" t="inlineStr">
         <is>
-          <t>WB-03</t>
+          <t>WB-03, WB-10</t>
         </is>
       </c>
     </row>
@@ -9463,7 +9463,7 @@
       </c>
       <c r="Q130" s="10" t="inlineStr">
         <is>
-          <t>WB-03, WB-05</t>
+          <t>WB-03, WB-05, WB-10</t>
         </is>
       </c>
     </row>
@@ -9528,7 +9528,7 @@
       </c>
       <c r="Q131" s="10" t="inlineStr">
         <is>
-          <t>WB-09</t>
+          <t>WB-09, WB-10</t>
         </is>
       </c>
     </row>
@@ -9911,7 +9911,7 @@
       <c r="M137" s="7" t="inlineStr"/>
       <c r="N137" s="8" t="inlineStr"/>
       <c r="O137" s="10" t="inlineStr"/>
-      <c r="P137" s="12" t="inlineStr">
+      <c r="P137" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -9983,7 +9983,7 @@
       </c>
       <c r="Q138" s="10" t="inlineStr">
         <is>
-          <t>IA-01</t>
+          <t>IA-01, IA-32</t>
         </is>
       </c>
     </row>
@@ -10041,7 +10041,7 @@
       <c r="M139" s="7" t="inlineStr"/>
       <c r="N139" s="8" t="inlineStr"/>
       <c r="O139" s="10" t="inlineStr"/>
-      <c r="P139" s="12" t="inlineStr">
+      <c r="P139" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -10113,7 +10113,7 @@
       </c>
       <c r="Q140" s="10" t="inlineStr">
         <is>
-          <t>IA-03</t>
+          <t>IA-03, IA-32</t>
         </is>
       </c>
     </row>
@@ -10308,7 +10308,7 @@
       </c>
       <c r="Q143" s="10" t="inlineStr">
         <is>
-          <t>IA-06</t>
+          <t>IA-06, IA-26</t>
         </is>
       </c>
     </row>
@@ -10373,7 +10373,7 @@
       </c>
       <c r="Q144" s="10" t="inlineStr">
         <is>
-          <t>IA-06, IA-22</t>
+          <t>IA-06, IA-22, IA-26</t>
         </is>
       </c>
     </row>
@@ -10438,7 +10438,7 @@
       </c>
       <c r="Q145" s="10" t="inlineStr">
         <is>
-          <t>IA-05</t>
+          <t>IA-05, IA-27</t>
         </is>
       </c>
     </row>
@@ -10691,14 +10691,14 @@
       <c r="M149" s="7" t="inlineStr"/>
       <c r="N149" s="8" t="inlineStr"/>
       <c r="O149" s="10" t="inlineStr"/>
-      <c r="P149" s="12" t="inlineStr">
-        <is>
-          <t>Connaissance</t>
+      <c r="P149" s="11" t="inlineStr">
+        <is>
+          <t>Compétence</t>
         </is>
       </c>
       <c r="Q149" s="10" t="inlineStr">
         <is>
-          <t>IA-08</t>
+          <t>IA-08, IA-29</t>
         </is>
       </c>
     </row>
@@ -10828,7 +10828,7 @@
       </c>
       <c r="Q151" s="10" t="inlineStr">
         <is>
-          <t>IA-10, IA-19</t>
+          <t>IA-10, IA-19, IA-28</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11088,7 @@
       </c>
       <c r="Q155" s="10" t="inlineStr">
         <is>
-          <t>IA-11, IA-17</t>
+          <t>IA-11, IA-17, IA-33</t>
         </is>
       </c>
     </row>
@@ -11218,7 +11218,7 @@
       </c>
       <c r="Q157" s="10" t="inlineStr">
         <is>
-          <t>IA-12</t>
+          <t>IA-12, IA-31</t>
         </is>
       </c>
     </row>
@@ -11283,7 +11283,7 @@
       </c>
       <c r="Q158" s="10" t="inlineStr">
         <is>
-          <t>IA-12, IA-15</t>
+          <t>IA-12, IA-15, IA-31</t>
         </is>
       </c>
     </row>
@@ -11348,7 +11348,7 @@
       </c>
       <c r="Q159" s="10" t="inlineStr">
         <is>
-          <t>IA-12, IA-16</t>
+          <t>IA-12, IA-16, IA-31</t>
         </is>
       </c>
     </row>
@@ -11471,7 +11471,7 @@
       <c r="M161" s="7" t="inlineStr"/>
       <c r="N161" s="8" t="inlineStr"/>
       <c r="O161" s="10" t="inlineStr"/>
-      <c r="P161" s="12" t="inlineStr">
+      <c r="P161" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -11536,7 +11536,7 @@
       <c r="M162" s="7" t="inlineStr"/>
       <c r="N162" s="8" t="inlineStr"/>
       <c r="O162" s="10" t="inlineStr"/>
-      <c r="P162" s="12" t="inlineStr">
+      <c r="P162" s="13" t="inlineStr">
         <is>
           <t>Connaissance</t>
         </is>
@@ -11608,7 +11608,7 @@
       </c>
       <c r="Q163" s="10" t="inlineStr">
         <is>
-          <t>IA-14, IA-25</t>
+          <t>IA-14, IA-25, IA-30</t>
         </is>
       </c>
     </row>

</xml_diff>